<commit_message>
Refine timetable layout, implement strict print format, and add PSNA branding
</commit_message>
<xml_diff>
--- a/sample_timetable_data.xlsx
+++ b/sample_timetable_data.xlsx
@@ -3,8 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Teachers" sheetId="1" r:id="rId1"/>
-    <sheet name="Subjects" sheetId="2" r:id="rId2"/>
+    <sheet name="Allocations" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -398,186 +397,518 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:M12"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" customWidth="1"/>
+    <col min="7" max="7" width="10.83203125" customWidth="1"/>
+    <col min="8" max="8" width="10.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" customWidth="1"/>
+    <col min="11" max="11" width="8.83203125" customWidth="1"/>
+    <col min="12" max="12" width="15.83203125" customWidth="1"/>
+    <col min="13" max="13" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Name</v>
+        <v>SEMESTER</v>
       </c>
       <c r="B1" t="str">
-        <v>Department</v>
+        <v>SUB.COD</v>
       </c>
       <c r="C1" t="str">
-        <v>Workload</v>
+        <v>SUBJECT NAME</v>
+      </c>
+      <c r="D1" t="str">
+        <v>A</v>
+      </c>
+      <c r="E1" t="str">
+        <v>B</v>
+      </c>
+      <c r="F1" t="str">
+        <v>C</v>
+      </c>
+      <c r="G1" t="str">
+        <v>D</v>
+      </c>
+      <c r="H1" t="str">
+        <v>E</v>
+      </c>
+      <c r="I1" t="str">
+        <v>No of Section</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Sub Hand Dept</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Tutorial</v>
+      </c>
+      <c r="L1" t="str">
+        <v>No.of Hours allotted</v>
+      </c>
+      <c r="M1" t="str">
+        <v>SATURDAY</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Dr. Alice Smith</v>
+        <v>II CSE</v>
       </c>
       <c r="B2" t="str">
-        <v>Computer Science</v>
-      </c>
-      <c r="C2">
-        <v>12</v>
+        <v>HS2221</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Communicative English</v>
+      </c>
+      <c r="D2" t="str">
+        <v>HAJIRA B</v>
+      </c>
+      <c r="E2" t="str">
+        <v>M.KSUBA</v>
+      </c>
+      <c r="F2" t="str">
+        <v>HAJIRA B</v>
+      </c>
+      <c r="G2" t="str">
+        <v>M.KSUBA</v>
+      </c>
+      <c r="H2" t="str">
+        <v>VIJAY</v>
+      </c>
+      <c r="I2">
+        <v>5</v>
+      </c>
+      <c r="J2" t="str">
+        <v>ENG</v>
+      </c>
+      <c r="K2" t="str">
+        <v>NO</v>
+      </c>
+      <c r="L2">
+        <v>2</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Prof. Bob Jones</v>
+        <v>II CSE</v>
       </c>
       <c r="B3" t="str">
-        <v>Electronics</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
+        <v>MA2224</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Probability, Statistics and Linear Algebra</v>
+      </c>
+      <c r="D3" t="str">
+        <v>M1</v>
+      </c>
+      <c r="E3" t="str">
+        <v>M2</v>
+      </c>
+      <c r="F3" t="str">
+        <v>M3</v>
+      </c>
+      <c r="G3" t="str">
+        <v>M4</v>
+      </c>
+      <c r="H3" t="str">
+        <v>M5</v>
+      </c>
+      <c r="I3">
+        <v>5</v>
+      </c>
+      <c r="J3" t="str">
+        <v>MAT</v>
+      </c>
+      <c r="K3" t="str">
+        <v>YES</v>
+      </c>
+      <c r="L3">
+        <v>5</v>
+      </c>
+      <c r="M3">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Ms. Carol White</v>
+        <v>II CSE</v>
       </c>
       <c r="B4" t="str">
-        <v>Mathematics</v>
-      </c>
-      <c r="C4">
-        <v>14</v>
+        <v>PH2221</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Quantum Physics</v>
+      </c>
+      <c r="D4" t="str">
+        <v>P1</v>
+      </c>
+      <c r="E4" t="str">
+        <v>P2</v>
+      </c>
+      <c r="F4" t="str">
+        <v>P3</v>
+      </c>
+      <c r="G4" t="str">
+        <v>P4</v>
+      </c>
+      <c r="H4" t="str">
+        <v>P5</v>
+      </c>
+      <c r="I4">
+        <v>5</v>
+      </c>
+      <c r="J4" t="str">
+        <v>PHY</v>
+      </c>
+      <c r="K4" t="str">
+        <v>NO</v>
+      </c>
+      <c r="L4">
+        <v>4</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Dr. David Black</v>
+        <v>II CSE</v>
       </c>
       <c r="B5" t="str">
-        <v>Physics</v>
-      </c>
-      <c r="C5">
-        <v>8</v>
+        <v>CS2221</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Programming in C</v>
+      </c>
+      <c r="D5" t="str">
+        <v>AJ</v>
+      </c>
+      <c r="E5" t="str">
+        <v>LED</v>
+      </c>
+      <c r="F5" t="str">
+        <v>NI</v>
+      </c>
+      <c r="G5" t="str">
+        <v>TD</v>
+      </c>
+      <c r="H5" t="str">
+        <v>MK</v>
+      </c>
+      <c r="I5">
+        <v>5</v>
+      </c>
+      <c r="J5" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="K5" t="str">
+        <v>NO</v>
+      </c>
+      <c r="L5">
+        <v>4</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>II CSE</v>
+      </c>
+      <c r="B6" t="str">
+        <v>GE2281</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Engineering Practice Laboratory</v>
+      </c>
+      <c r="D6" t="str">
+        <v>EP1</v>
+      </c>
+      <c r="E6" t="str">
+        <v>EP2</v>
+      </c>
+      <c r="F6" t="str">
+        <v>EP3</v>
+      </c>
+      <c r="G6" t="str">
+        <v>EP4</v>
+      </c>
+      <c r="H6" t="str">
+        <v>EP5</v>
+      </c>
+      <c r="I6">
+        <v>5</v>
+      </c>
+      <c r="J6" t="str">
+        <v>MECH/ECE</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>4</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>II CSE</v>
+      </c>
+      <c r="B7" t="str">
+        <v>CS2281</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Programming in C Laboratory</v>
+      </c>
+      <c r="D7" t="str">
+        <v>AJ</v>
+      </c>
+      <c r="E7" t="str">
+        <v>LED</v>
+      </c>
+      <c r="F7" t="str">
+        <v>NI</v>
+      </c>
+      <c r="G7" t="str">
+        <v>TD</v>
+      </c>
+      <c r="H7" t="str">
+        <v>MK</v>
+      </c>
+      <c r="I7">
+        <v>5</v>
+      </c>
+      <c r="J7" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>3</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>IV CSE</v>
+      </c>
+      <c r="B8" t="str">
+        <v>CS2411</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Theory of Computation</v>
+      </c>
+      <c r="D8" t="str">
+        <v>CS</v>
+      </c>
+      <c r="E8" t="str">
+        <v>ND</v>
+      </c>
+      <c r="F8" t="str">
+        <v>DS</v>
+      </c>
+      <c r="G8" t="str">
+        <v>NJ</v>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8">
+        <v>4</v>
+      </c>
+      <c r="J8" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="K8" t="str">
+        <v>NO</v>
+      </c>
+      <c r="L8">
+        <v>4</v>
+      </c>
+      <c r="M8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>IV CSE</v>
+      </c>
+      <c r="B9" t="str">
+        <v>CS2412</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Database Management Systems</v>
+      </c>
+      <c r="D9" t="str">
+        <v>VNK</v>
+      </c>
+      <c r="E9" t="str">
+        <v>SSP</v>
+      </c>
+      <c r="F9" t="str">
+        <v>RS</v>
+      </c>
+      <c r="G9" t="str">
+        <v>NPP</v>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9">
+        <v>4</v>
+      </c>
+      <c r="J9" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="K9" t="str">
+        <v>NO</v>
+      </c>
+      <c r="L9">
+        <v>4</v>
+      </c>
+      <c r="M9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>IV CSE</v>
+      </c>
+      <c r="B10" t="str">
+        <v>CS2413</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Computer Networks</v>
+      </c>
+      <c r="D10" t="str">
+        <v>GIM</v>
+      </c>
+      <c r="E10" t="str">
+        <v>LHL</v>
+      </c>
+      <c r="F10" t="str">
+        <v>SAF</v>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10">
+        <v>3</v>
+      </c>
+      <c r="J10" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="K10" t="str">
+        <v>NO</v>
+      </c>
+      <c r="L10">
+        <v>4</v>
+      </c>
+      <c r="M10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>VI CSE</v>
+      </c>
+      <c r="B11" t="str">
+        <v>CS2611</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Cryptography and Cyber Security</v>
+      </c>
+      <c r="D11" t="str">
+        <v>MST</v>
+      </c>
+      <c r="E11" t="str">
+        <v>GM</v>
+      </c>
+      <c r="F11" t="str">
+        <v>VP</v>
+      </c>
+      <c r="G11" t="str">
+        <v>ND</v>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11">
+        <v>4</v>
+      </c>
+      <c r="J11" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="K11" t="str">
+        <v>NO</v>
+      </c>
+      <c r="L11">
+        <v>4</v>
+      </c>
+      <c r="M11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>VI CSE</v>
+      </c>
+      <c r="B12" t="str">
+        <v>CS2612</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Internet of Things</v>
+      </c>
+      <c r="D12" t="str">
+        <v>ATP</v>
+      </c>
+      <c r="E12" t="str">
+        <v>SSB</v>
+      </c>
+      <c r="F12" t="str">
+        <v>DS</v>
+      </c>
+      <c r="G12" t="str">
+        <v>MJ</v>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12">
+        <v>4</v>
+      </c>
+      <c r="J12" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="K12" t="str">
+        <v>NO</v>
+      </c>
+      <c r="L12">
+        <v>3</v>
+      </c>
+      <c r="M12">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D7"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="8.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Code</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Name</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Type</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Credits</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>CS101</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Introduction to Programming</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Lecture</v>
-      </c>
-      <c r="D2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>CS102</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Data Structures &amp; Algorithms</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Lecture</v>
-      </c>
-      <c r="D3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>CS101L</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Programming Lab</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Lab</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>CS102L</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Data Structures Lab</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Lab</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>MA101</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Calculus I</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Lecture</v>
-      </c>
-      <c r="D6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>PH101</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Applied Physics</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Lecture</v>
-      </c>
-      <c r="D7">
-        <v>3</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>